<commit_message>
Corrida | SFE-MOTT | 2026-06-17 12:06:49.198365
</commit_message>
<xml_diff>
--- a/indicadores/SFE-MOTT_out.xlsx
+++ b/indicadores/SFE-MOTT_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="382">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Transferencia de motos usadas en la provincia de Santa Fe</t>
+    <t xml:space="preserve">Transferencia de motos usadas</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -74,6 +74,12 @@
     <t xml:space="preserve">td1coef</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provincia de Santa Fe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -107,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">08/06/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1656,9 +1662,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -1669,7 +1679,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -1683,7 +1693,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
@@ -1699,7 +1709,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -1727,7 +1737,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -1741,7 +1751,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
@@ -1769,7 +1779,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -1783,7 +1793,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -1797,7 +1807,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -1811,7 +1821,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
@@ -1827,7 +1837,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -1841,7 +1851,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
@@ -1989,10 +1999,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -2005,10 +2015,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -2032,66 +2042,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="O1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="P1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="Q1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="R1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="S1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>1497</v>
@@ -2144,7 +2154,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>1299</v>
@@ -2201,7 +2211,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>1502</v>
@@ -2258,7 +2268,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>1237</v>
@@ -2315,7 +2325,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>1358</v>
@@ -2372,7 +2382,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>1197</v>
@@ -2429,7 +2439,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>1311</v>
@@ -2486,7 +2496,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>1439</v>
@@ -2543,7 +2553,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>1504</v>
@@ -2600,7 +2610,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>1642</v>
@@ -2657,7 +2667,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>1776</v>
@@ -2714,7 +2724,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>1536</v>
@@ -2771,7 +2781,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>1841</v>
@@ -2830,7 +2840,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>2033</v>
@@ -2889,7 +2899,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>1897</v>
@@ -2948,7 +2958,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>2352</v>
@@ -3007,7 +3017,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>2239</v>
@@ -3066,7 +3076,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>1839</v>
@@ -3125,7 +3135,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>2106</v>
@@ -3184,7 +3194,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>2077</v>
@@ -3243,7 +3253,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>2231</v>
@@ -3302,7 +3312,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>2279</v>
@@ -3361,7 +3371,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>1968</v>
@@ -3420,7 +3430,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>1809</v>
@@ -3479,7 +3489,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>2011</v>
@@ -3538,7 +3548,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>1914</v>
@@ -3597,7 +3607,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>2042</v>
@@ -3656,7 +3666,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>2018</v>
@@ -3715,7 +3725,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>1910</v>
@@ -3774,7 +3784,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>1905</v>
@@ -3833,7 +3843,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>2042</v>
@@ -3892,7 +3902,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>1986</v>
@@ -3951,7 +3961,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>2235</v>
@@ -4010,7 +4020,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>2199</v>
@@ -4069,7 +4079,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>2104</v>
@@ -4128,7 +4138,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>2055</v>
@@ -4187,7 +4197,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>2253</v>
@@ -4246,7 +4256,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>2186</v>
@@ -4305,7 +4315,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>2505</v>
@@ -4364,7 +4374,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>2445</v>
@@ -4423,7 +4433,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>2169</v>
@@ -4482,7 +4492,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>2282</v>
@@ -4541,7 +4551,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>2331</v>
@@ -4600,7 +4610,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>2617</v>
@@ -4659,7 +4669,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>2809</v>
@@ -4718,7 +4728,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>2420</v>
@@ -4777,7 +4787,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>2930</v>
@@ -4836,7 +4846,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>2791</v>
@@ -4895,7 +4905,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>2836</v>
@@ -4954,7 +4964,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>2755</v>
@@ -5013,7 +5023,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>2997</v>
@@ -5072,7 +5082,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>2655</v>
@@ -5131,7 +5141,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>3205</v>
@@ -5190,7 +5200,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>2708</v>
@@ -5249,7 +5259,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>2780</v>
@@ -5308,7 +5318,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>3266</v>
@@ -5367,7 +5377,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>3500</v>
@@ -5426,7 +5436,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>3310</v>
@@ -5485,7 +5495,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>3333</v>
@@ -5544,7 +5554,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>3236</v>
@@ -5603,7 +5613,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>3156</v>
@@ -5662,7 +5672,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>2763</v>
@@ -5721,7 +5731,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>3596</v>
@@ -5780,7 +5790,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>2919</v>
@@ -5839,7 +5849,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>3564</v>
@@ -5898,7 +5908,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>3019</v>
@@ -5957,7 +5967,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>3100</v>
@@ -6016,7 +6026,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>3518</v>
@@ -6075,7 +6085,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>2981</v>
@@ -6134,7 +6144,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>3277</v>
@@ -6193,7 +6203,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>3075</v>
@@ -6252,7 +6262,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>2505</v>
@@ -6311,7 +6321,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>3176</v>
@@ -6370,7 +6380,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>2687</v>
@@ -6429,7 +6439,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>3226</v>
@@ -6488,7 +6498,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>3380</v>
@@ -6547,7 +6557,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>3614</v>
@@ -6606,7 +6616,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>2808</v>
@@ -6665,7 +6675,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>3277</v>
@@ -6724,7 +6734,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>3392</v>
@@ -6783,7 +6793,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>3517</v>
@@ -6842,7 +6852,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>3550</v>
@@ -6901,7 +6911,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>3092</v>
@@ -6960,7 +6970,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>2944</v>
@@ -7019,7 +7029,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>3356</v>
@@ -7078,7 +7088,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>3060</v>
@@ -7137,7 +7147,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>2843</v>
@@ -7196,7 +7206,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>2892</v>
@@ -7255,7 +7265,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>3297</v>
@@ -7314,7 +7324,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>2936</v>
@@ -7373,7 +7383,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>3591</v>
@@ -7432,7 +7442,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>3215</v>
@@ -7491,7 +7501,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>3810</v>
@@ -7550,7 +7560,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>3820</v>
@@ -7609,7 +7619,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>3207</v>
@@ -7668,7 +7678,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>3353</v>
@@ -7727,7 +7737,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>3358</v>
@@ -7786,7 +7796,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>2915</v>
@@ -7845,7 +7855,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>3452</v>
@@ -7904,7 +7914,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>3640</v>
@@ -7963,7 +7973,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>3192</v>
@@ -8022,7 +8032,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>3519</v>
@@ -8081,7 +8091,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>3775</v>
@@ -8140,7 +8150,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>3347</v>
@@ -8199,7 +8209,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>3903</v>
@@ -8258,7 +8268,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>3781</v>
@@ -8317,7 +8327,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>3431</v>
@@ -8376,7 +8386,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>3082</v>
@@ -8435,7 +8445,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>3137</v>
@@ -8494,7 +8504,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>2886</v>
@@ -8553,7 +8563,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>3424</v>
@@ -8612,7 +8622,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>2858</v>
@@ -8671,7 +8681,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>2860</v>
@@ -8730,7 +8740,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>2164</v>
@@ -8789,7 +8799,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>2446</v>
@@ -8848,7 +8858,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>2986</v>
@@ -8907,7 +8917,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>3185</v>
@@ -8966,7 +8976,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>2924</v>
@@ -9025,7 +9035,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>2921</v>
@@ -9084,7 +9094,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>3049</v>
@@ -9143,7 +9153,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>3011</v>
@@ -9202,7 +9212,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>2660</v>
@@ -9261,7 +9271,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>3610</v>
@@ -9320,7 +9330,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>2727</v>
@@ -9379,7 +9389,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>2894</v>
@@ -9438,7 +9448,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>2637</v>
@@ -9497,7 +9507,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>3110</v>
@@ -9556,7 +9566,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>3405</v>
@@ -9615,7 +9625,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>3472</v>
@@ -9674,7 +9684,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>3261</v>
@@ -9733,7 +9743,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>3289</v>
@@ -9792,7 +9802,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>3001</v>
@@ -9851,7 +9861,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>3441</v>
@@ -9910,7 +9920,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>2931</v>
@@ -9969,7 +9979,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>3497</v>
@@ -10028,7 +10038,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>3282</v>
@@ -10087,7 +10097,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>3111</v>
@@ -10146,7 +10156,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>2701</v>
@@ -10205,7 +10215,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>3311</v>
@@ -10264,7 +10274,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>3555</v>
@@ -10323,7 +10333,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>3606</v>
@@ -10382,7 +10392,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>3928</v>
@@ -10441,7 +10451,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>3192</v>
@@ -10500,7 +10510,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>2903</v>
@@ -10559,7 +10569,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>3739</v>
@@ -10618,7 +10628,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>3679</v>
@@ -10677,7 +10687,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>3516</v>
@@ -10736,7 +10746,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>3654</v>
@@ -10795,7 +10805,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>4138</v>
@@ -10854,7 +10864,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>3155</v>
@@ -10913,7 +10923,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>3777</v>
@@ -10972,7 +10982,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>3838</v>
@@ -11031,7 +11041,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>3858</v>
@@ -11090,7 +11100,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>3952</v>
@@ -11149,7 +11159,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>3381</v>
@@ -11208,7 +11218,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>3281</v>
@@ -11267,7 +11277,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>3726</v>
@@ -11326,7 +11336,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>3272</v>
@@ -11385,7 +11395,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>2523</v>
@@ -11444,7 +11454,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>540</v>
@@ -11503,7 +11513,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>2586</v>
@@ -11562,7 +11572,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>4032</v>
@@ -11621,7 +11631,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>4820</v>
@@ -11680,7 +11690,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>4940</v>
@@ -11739,7 +11749,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>4790</v>
@@ -11798,7 +11808,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>4904</v>
@@ -11857,7 +11867,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>4524</v>
@@ -11916,7 +11926,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>3924</v>
@@ -11975,7 +11985,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>3917</v>
@@ -12034,7 +12044,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>3812</v>
@@ -12093,7 +12103,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>4704</v>
@@ -12152,7 +12162,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>3833</v>
@@ -12211,7 +12221,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>3139</v>
@@ -12270,7 +12280,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>4323</v>
@@ -12329,7 +12339,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>4448</v>
@@ -12388,7 +12398,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>4474</v>
@@ -12447,7 +12457,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>5033</v>
@@ -12506,7 +12516,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>4270</v>
@@ -12565,7 +12575,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>4572</v>
@@ -12624,7 +12634,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>4504</v>
@@ -12683,7 +12693,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>3795</v>
@@ -12742,7 +12752,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>4067</v>
@@ -12801,7 +12811,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>4807</v>
@@ -12860,7 +12870,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>4459</v>
@@ -12919,7 +12929,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>4833</v>
@@ -12978,7 +12988,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>4611</v>
@@ -13037,7 +13047,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>5009</v>
@@ -13096,7 +13106,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>5275</v>
@@ -13155,7 +13165,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>5519</v>
@@ -13214,7 +13224,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>4580</v>
@@ -13273,7 +13283,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>4892</v>
@@ -13332,7 +13342,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>4227</v>
@@ -13391,7 +13401,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>4916</v>
@@ -13450,7 +13460,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>4065</v>
@@ -13509,7 +13519,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>5424</v>
@@ -13568,7 +13578,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>4601</v>
@@ -13627,7 +13637,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>5077</v>
@@ -13686,7 +13696,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>4324</v>
@@ -13745,7 +13755,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>5110</v>
@@ -13804,7 +13814,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>5564</v>
@@ -13863,7 +13873,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>5354</v>
@@ -13922,7 +13932,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>5388</v>
@@ -13981,7 +13991,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>5352</v>
@@ -14040,7 +14050,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>4743</v>
@@ -14099,7 +14109,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>4927</v>
@@ -14158,7 +14168,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>4444</v>
@@ -14217,7 +14227,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>4413</v>
@@ -14276,7 +14286,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>5322</v>
@@ -14335,7 +14345,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>5612</v>
@@ -14394,7 +14404,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>4285</v>
@@ -14453,7 +14463,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>6449</v>
@@ -14512,7 +14522,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>6481</v>
@@ -14571,7 +14581,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>6597</v>
@@ -14630,7 +14640,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>6740</v>
@@ -14689,7 +14699,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>5747</v>
@@ -14748,7 +14758,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>5678</v>
@@ -14807,7 +14817,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>6376</v>
@@ -14866,7 +14876,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>5754</v>
@@ -14925,7 +14935,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>5432</v>
@@ -14984,7 +14994,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>5870</v>
@@ -15043,7 +15053,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B222" s="2" t="n">
         <v>5918</v>
@@ -15102,7 +15112,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B223" s="2" t="n">
         <v>5234</v>
@@ -15161,7 +15171,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B224" s="2" t="n">
         <v>5887</v>
@@ -15220,7 +15230,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B225" s="2" t="n">
         <v>5734</v>
@@ -15279,7 +15289,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B226" s="2" t="n">
         <v>6314</v>
@@ -15338,7 +15348,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B227" s="2" t="n">
         <v>6322</v>
@@ -15397,7 +15407,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B228" s="2" t="n">
         <v>5161</v>
@@ -15456,7 +15466,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B229" s="2" t="n">
         <v>5917</v>
@@ -15515,7 +15525,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B230" s="2" t="n">
         <v>5911</v>
@@ -15574,7 +15584,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B231" s="2" t="n">
         <v>5337</v>
@@ -15633,7 +15643,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B232" s="2" t="n">
         <v>6265</v>
@@ -15692,7 +15702,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B233" s="2" t="n">
         <v>6124</v>
@@ -15751,7 +15761,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B234" s="2" t="n">
         <v>5724</v>
@@ -15810,7 +15820,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B235" s="2"/>
       <c r="C235" s="3" t="n">
@@ -15843,7 +15853,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B236" s="2"/>
       <c r="C236" s="3" t="n">
@@ -15876,7 +15886,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B237" s="2"/>
       <c r="C237" s="3" t="n">
@@ -15909,7 +15919,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B238" s="2"/>
       <c r="C238" s="3" t="n">
@@ -15942,7 +15952,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B239" s="2"/>
       <c r="C239" s="3" t="n">
@@ -15975,7 +15985,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B240" s="2"/>
       <c r="C240" s="3" t="n">
@@ -16008,7 +16018,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B241" s="2"/>
       <c r="C241" s="3" t="n">
@@ -16041,7 +16051,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B242" s="2"/>
       <c r="C242" s="3" t="n">
@@ -16074,7 +16084,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B243" s="2"/>
       <c r="C243" s="3" t="n">
@@ -16107,7 +16117,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B244" s="2"/>
       <c r="C244" s="3" t="n">
@@ -16140,7 +16150,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B245" s="2"/>
       <c r="C245" s="3" t="n">
@@ -16173,7 +16183,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B246" s="2"/>
       <c r="C246" s="3" t="n">
@@ -16206,7 +16216,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B247" s="2"/>
       <c r="C247" s="3"/>
@@ -16229,7 +16239,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B248" s="2"/>
       <c r="C248" s="3"/>
@@ -16252,7 +16262,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B249" s="2"/>
       <c r="C249" s="3"/>
@@ -16275,7 +16285,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B250" s="2"/>
       <c r="C250" s="3"/>
@@ -16298,7 +16308,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B251" s="2"/>
       <c r="C251" s="3"/>
@@ -16321,7 +16331,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B252" s="2"/>
       <c r="C252" s="3"/>
@@ -16344,7 +16354,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B253" s="2"/>
       <c r="C253" s="3"/>
@@ -16367,7 +16377,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B254" s="2"/>
       <c r="C254" s="3"/>
@@ -16390,7 +16400,7 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B255" s="2"/>
       <c r="C255" s="3"/>
@@ -16413,7 +16423,7 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B256" s="2"/>
       <c r="C256" s="3"/>
@@ -16436,7 +16446,7 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B257" s="2"/>
       <c r="C257" s="3"/>
@@ -16459,7 +16469,7 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B258" s="2"/>
       <c r="C258" s="3"/>
@@ -16482,7 +16492,7 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B259" s="2"/>
       <c r="C259" s="3"/>
@@ -16505,7 +16515,7 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B260" s="2"/>
       <c r="C260" s="3"/>
@@ -16528,7 +16538,7 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B261" s="2"/>
       <c r="C261" s="3"/>
@@ -16551,7 +16561,7 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B262" s="2"/>
       <c r="C262" s="3"/>
@@ -16574,7 +16584,7 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B263" s="2"/>
       <c r="C263" s="3"/>
@@ -16597,7 +16607,7 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B264" s="2"/>
       <c r="C264" s="3"/>
@@ -16620,7 +16630,7 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B265" s="2"/>
       <c r="C265" s="3"/>
@@ -16643,7 +16653,7 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B266" s="2"/>
       <c r="C266" s="3"/>
@@ -16666,7 +16676,7 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B267" s="2"/>
       <c r="C267" s="3"/>
@@ -16689,7 +16699,7 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B268" s="2"/>
       <c r="C268" s="3"/>
@@ -16712,7 +16722,7 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B269" s="2"/>
       <c r="C269" s="3"/>
@@ -16735,7 +16745,7 @@
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B270" s="2"/>
       <c r="C270" s="3"/>
@@ -16758,7 +16768,7 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B271" s="2"/>
       <c r="C271" s="3"/>
@@ -16781,7 +16791,7 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B272" s="2"/>
       <c r="C272" s="3"/>
@@ -16804,7 +16814,7 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B273" s="2"/>
       <c r="C273" s="3"/>
@@ -16827,7 +16837,7 @@
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B274" s="2"/>
       <c r="C274" s="3"/>
@@ -16850,7 +16860,7 @@
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B275" s="2"/>
       <c r="C275" s="3"/>
@@ -16873,7 +16883,7 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B276" s="2"/>
       <c r="C276" s="3"/>
@@ -16896,7 +16906,7 @@
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B277" s="2"/>
       <c r="C277" s="3"/>
@@ -16919,7 +16929,7 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B278" s="2"/>
       <c r="C278" s="3"/>
@@ -16942,7 +16952,7 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B279" s="2"/>
       <c r="C279" s="3"/>
@@ -16965,7 +16975,7 @@
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B280" s="2"/>
       <c r="C280" s="3"/>
@@ -16988,7 +16998,7 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B281" s="2"/>
       <c r="C281" s="3"/>
@@ -17011,7 +17021,7 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B282" s="2"/>
       <c r="C282" s="3"/>
@@ -17034,7 +17044,7 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B283" s="2"/>
       <c r="C283" s="3"/>
@@ -17057,7 +17067,7 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B284" s="2"/>
       <c r="C284" s="3"/>
@@ -17080,7 +17090,7 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B285" s="2"/>
       <c r="C285" s="3"/>
@@ -17103,7 +17113,7 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B286" s="2"/>
       <c r="C286" s="3"/>
@@ -17126,7 +17136,7 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B287" s="2"/>
       <c r="C287" s="3"/>
@@ -17149,7 +17159,7 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B288" s="2"/>
       <c r="C288" s="3"/>
@@ -17172,7 +17182,7 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B289" s="2"/>
       <c r="C289" s="3"/>
@@ -17206,97 +17216,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
     </row>
   </sheetData>
@@ -17320,7 +17330,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -17330,13 +17340,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>-0.0968151836844128</v>
@@ -17344,7 +17354,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>-0.0699737375874157</v>
@@ -17352,7 +17362,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>-0.0102520049253243</v>
@@ -17360,7 +17370,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0.0697463552884373</v>
@@ -17368,7 +17378,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0.130655890495955</v>
@@ -17376,7 +17386,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>0.197276554910285</v>
@@ -17384,7 +17394,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>0.258084290390461</v>
@@ -17392,7 +17402,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>0.286450389374061</v>
@@ -17400,7 +17410,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>0.353757052853121</v>
@@ -17408,7 +17418,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>0.4001009230359</v>
@@ -17416,7 +17426,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>0.270657808561006</v>
@@ -17424,7 +17434,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>0.12394090162617</v>
@@ -17432,7 +17442,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>0.102839927950213</v>
@@ -17440,7 +17450,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>0.045240756880869</v>
@@ -17448,7 +17458,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>-0.0802076634280899</v>
@@ -17456,7 +17466,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>-0.146787987684037</v>
@@ -17464,7 +17474,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>-0.133348415619871</v>
@@ -17472,7 +17482,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>-0.122194692412362</v>
@@ -17480,7 +17490,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>-0.131119907658964</v>

</xml_diff>